<commit_message>
Add generated_transfer_RIZ5.tvr with initial configuration and parameters
- Introduced a new transfer file `generated_transfer_RIZ5.tvr`
- Configured multiple sections with parameters for RIZ5 and MXZ5
- Included time intervals and limits for various operations
- Set specific values for each section to define behavior and constraints
</commit_message>
<xml_diff>
--- a/generated_transfer_RIZ5.xlsx
+++ b/generated_transfer_RIZ5.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW8"/>
+  <dimension ref="A1:BW11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,7 +808,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>961</v>
+        <v>985</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -818,11 +818,11 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>963</v>
+        <v>987</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>963</v>
+        <v>987</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
@@ -860,7 +860,7 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -902,7 +902,7 @@
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr">
         <is>
-          <t>20;600</t>
+          <t>12;600</t>
         </is>
       </c>
       <c r="BC2" t="n">
@@ -926,12 +926,12 @@
       </c>
       <c r="BH2" t="inlineStr">
         <is>
-          <t>105435;289917.5;86716.15; (20)</t>
+          <t>99429.1666666667;266637.5;84703.0416666667; (12)</t>
         </is>
       </c>
       <c r="BI2" t="inlineStr">
         <is>
-          <t>1;1;0.1;0.5</t>
+          <t>1;2;0.1;0.5</t>
         </is>
       </c>
       <c r="BJ2" t="inlineStr"/>
@@ -941,20 +941,22 @@
       </c>
       <c r="BM2" t="inlineStr">
         <is>
-          <t>2025.05.14 18:12:00</t>
+          <t>2025.04.21 09:00:00</t>
         </is>
       </c>
       <c r="BN2" t="inlineStr">
         <is>
-          <t>09:00:20-10:00:00 10:01:00-11:00:00 11:01:00-12:00:00 12:01:00-13:00:00 13:01:00-13:59:00 14:01:00-15:00:00 15:01:00-16:00:00 16:01:00-17:00:00 17:01:00-18:00:00 18:01:00-19:00:00 19:01:00-20:00:00 20:01:00-21:00:00 21:01:00-22:00:00 22:01:00-23:00:00 23:01:00-23:50:00</t>
+          <t>09:00:20-09:10:00 09:11:00-10:10:00 10:11:00-11:10:00 11:11:00-12:10:00 12:11:00-13:10:00 13:11:00-14:10:00 14:11:00-15:10:00 15:11:00-16:10:00 16:11:00-17:10:00 17:11:00-18:10:00 18:11:00-19:10:00 19:11:00-20:10:00 20:11:00-21:10:00 21:11:00-22:10:00 22:11:00-23:10:00 23:11:00-23:50:00</t>
         </is>
       </c>
       <c r="BO2" t="inlineStr">
         <is>
-          <t>09:00:20-10:00:00 10:01:00-11:00:00 11:01:00-12:00:00 12:01:00-13:00:00 13:01:00-13:59:00 14:01:00-15:00:00 15:01:00-16:00:00 16:01:00-17:00:00 17:01:00-18:00:00 18:01:00-19:00:00 19:01:00-20:00:00 20:01:00-21:00:00 21:01:00-22:00:00 22:01:00-23:00:00 23:01:00-23:50:00</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr"/>
+          <t>09:00:20-09:10:00 09:11:00-10:10:00 10:11:00-11:10:00 11:11:00-12:10:00 12:11:00-13:10:00 13:11:00-14:10:00 14:11:00-15:10:00 15:11:00-16:10:00 16:11:00-17:10:00 17:11:00-18:10:00 18:11:00-19:10:00 19:11:00-20:10:00 20:11:00-21:10:00 21:11:00-22:10:00 22:11:00-23:10:00 23:11:00-23:50:00</t>
+        </is>
+      </c>
+      <c r="BP2" t="n">
+        <v>98</v>
+      </c>
       <c r="BQ2" t="inlineStr">
         <is>
           <t>5/1</t>
@@ -975,7 +977,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>962</v>
+        <v>986</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -985,11 +987,11 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>963</v>
+        <v>987</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>963</v>
+        <v>987</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -1023,7 +1025,7 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -1065,7 +1067,7 @@
       <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="inlineStr">
         <is>
-          <t>20;600</t>
+          <t>12;600</t>
         </is>
       </c>
       <c r="BC3" t="n">
@@ -1089,12 +1091,12 @@
       </c>
       <c r="BH3" t="inlineStr">
         <is>
-          <t>105479.25;290003.125;86700.575; (20)</t>
+          <t>99429.1666666667;266637.5;84703.0416666667; (12)</t>
         </is>
       </c>
       <c r="BI3" t="inlineStr">
         <is>
-          <t>1;1;0.1;0.5</t>
+          <t>1;2;0.1;0.5</t>
         </is>
       </c>
       <c r="BJ3" t="inlineStr"/>
@@ -1104,20 +1106,22 @@
       </c>
       <c r="BM3" t="inlineStr">
         <is>
-          <t>2025.05.14 18:12:00</t>
+          <t>2025.04.21 09:00:00</t>
         </is>
       </c>
       <c r="BN3" t="inlineStr">
         <is>
-          <t>09:00:20-10:00:00 10:01:00-11:00:00 11:01:00-12:00:00 12:01:00-13:00:00 13:01:00-13:59:00 14:01:00-15:00:00 15:01:00-16:00:00 16:01:00-17:00:00 17:01:00-18:00:00 18:01:00-19:00:00 19:01:00-20:00:00 20:01:00-21:00:00 21:01:00-22:00:00 22:01:00-23:00:00 23:01:00-23:50:00</t>
+          <t>09:00:20-09:10:00 09:11:00-10:10:00 10:11:00-11:10:00 11:11:00-12:10:00 12:11:00-13:10:00 13:11:00-14:10:00 14:11:00-15:10:00 15:11:00-16:10:00 16:11:00-17:10:00 17:11:00-18:10:00 18:11:00-19:10:00 19:11:00-20:10:00 20:11:00-21:10:00 21:11:00-22:10:00 22:11:00-23:10:00 23:11:00-23:50:00</t>
         </is>
       </c>
       <c r="BO3" t="inlineStr">
         <is>
-          <t>09:00:20-10:00:00 10:01:00-11:00:00 11:01:00-12:00:00 12:01:00-13:00:00 13:01:00-13:59:00 14:01:00-15:00:00 15:01:00-16:00:00 16:01:00-17:00:00 17:01:00-18:00:00 18:01:00-19:00:00 19:01:00-20:00:00 20:01:00-21:00:00 21:01:00-22:00:00 22:01:00-23:00:00 23:01:00-23:50:00</t>
-        </is>
-      </c>
-      <c r="BP3" t="inlineStr"/>
+          <t>09:00:20-09:10:00 09:11:00-10:10:00 10:11:00-11:10:00 11:11:00-12:10:00 12:11:00-13:10:00 13:11:00-14:10:00 14:11:00-15:10:00 15:11:00-16:10:00 16:11:00-17:10:00 17:11:00-18:10:00 18:11:00-19:10:00 19:11:00-20:10:00 20:11:00-21:10:00 21:11:00-22:10:00 22:11:00-23:10:00 23:11:00-23:50:00</t>
+        </is>
+      </c>
+      <c r="BP3" t="n">
+        <v>98</v>
+      </c>
       <c r="BQ3" t="inlineStr">
         <is>
           <t>5/1</t>
@@ -1138,17 +1142,17 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>963</v>
+        <v>987</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>964</v>
+        <v>988</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>964</v>
+        <v>988</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -1182,18 +1186,18 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>AKZ5</t>
+          <t>LKZ5</t>
         </is>
       </c>
       <c r="U4" t="n">
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>7</v>
+        <v>1.7</v>
       </c>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
@@ -1232,14 +1236,14 @@
       <c r="BA4" t="inlineStr"/>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>20;600</t>
+          <t>12;600</t>
         </is>
       </c>
       <c r="BC4" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="BE4" t="inlineStr">
         <is>
@@ -1249,19 +1253,15 @@
       <c r="BF4" t="n">
         <v>1</v>
       </c>
-      <c r="BG4" t="inlineStr">
-        <is>
-          <t>2;60</t>
-        </is>
-      </c>
+      <c r="BG4" t="inlineStr"/>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>105435;289925.625;86716.45;15674.3; (20)</t>
+          <t>99429.1666666667;266637.5;84703.9166666667;59901.2083333333; (12)</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
         <is>
-          <t>1;1;0.01;0.2</t>
+          <t>1;1;0.01;0.3</t>
         </is>
       </c>
       <c r="BJ4" t="inlineStr"/>
@@ -1269,7 +1269,7 @@
       <c r="BL4" t="inlineStr"/>
       <c r="BM4" t="inlineStr">
         <is>
-          <t>2025.05.13 11:12:00</t>
+          <t>2025.04.14 09:00:00</t>
         </is>
       </c>
       <c r="BN4" t="inlineStr">
@@ -1297,17 +1297,17 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>964</v>
+        <v>988</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>965</v>
+        <v>989</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>965</v>
+        <v>989</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -1341,18 +1341,18 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>AKZ5</t>
+          <t>LKZ5</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V5" t="n">
-        <v>7</v>
+        <v>1.7</v>
       </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -1383,22 +1383,22 @@
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
       <c r="AY5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AZ5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA5" t="inlineStr"/>
       <c r="BB5" t="inlineStr">
         <is>
-          <t>5;60</t>
+          <t>1;60</t>
         </is>
       </c>
       <c r="BC5" t="n">
-        <v>-0.001</v>
+        <v>-0.002</v>
       </c>
       <c r="BD5" t="n">
-        <v>-0.001</v>
+        <v>-0.002</v>
       </c>
       <c r="BE5" t="inlineStr">
         <is>
@@ -1411,12 +1411,12 @@
       <c r="BG5" t="inlineStr"/>
       <c r="BH5" t="inlineStr">
         <is>
-          <t>105175;289050;86697.8;15632.1; (5)</t>
+          <t>100210;269912.5;84904;60239.5; (1)</t>
         </is>
       </c>
       <c r="BI5" t="inlineStr">
         <is>
-          <t>1;1;0.01;0.2</t>
+          <t>1;2;0.2;0.3</t>
         </is>
       </c>
       <c r="BJ5" t="inlineStr"/>
@@ -1424,7 +1424,7 @@
       <c r="BL5" t="inlineStr"/>
       <c r="BM5" t="inlineStr">
         <is>
-          <t>2025.05.13 11:12:00</t>
+          <t>2025.04.14 09:00:00</t>
         </is>
       </c>
       <c r="BN5" t="inlineStr">
@@ -1438,7 +1438,11 @@
         </is>
       </c>
       <c r="BP5" t="inlineStr"/>
-      <c r="BQ5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="inlineStr"/>
       <c r="BT5" t="inlineStr"/>
@@ -1448,17 +1452,17 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>965</v>
+        <v>989</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>966</v>
+        <v>990</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>966</v>
+        <v>990</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -1492,7 +1496,7 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1534,11 +1538,11 @@
       <c r="BA6" t="inlineStr"/>
       <c r="BB6" t="inlineStr">
         <is>
-          <t>20;600</t>
+          <t>12;600</t>
         </is>
       </c>
       <c r="BC6" t="n">
-        <v>0.0001</v>
+        <v>0.001</v>
       </c>
       <c r="BD6" t="n">
         <v>0.0001</v>
@@ -1558,12 +1562,12 @@
       </c>
       <c r="BH6" t="inlineStr">
         <is>
-          <t>105435;289925.625;86716.45; (20)</t>
+          <t>99429.1666666667;266637.5;84703.0416666667; (12)</t>
         </is>
       </c>
       <c r="BI6" t="inlineStr">
         <is>
-          <t>1;1;0.01;0.2</t>
+          <t>1;1;0.01;0.3</t>
         </is>
       </c>
       <c r="BJ6" t="inlineStr"/>
@@ -1595,17 +1599,17 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>966</v>
+        <v>990</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>967</v>
+        <v>991</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>967</v>
+        <v>991</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -1693,12 +1697,12 @@
       <c r="BG7" t="inlineStr"/>
       <c r="BH7" t="inlineStr">
         <is>
-          <t>105187.5;105187.5; (2)</t>
+          <t>100345;100345; (2)</t>
         </is>
       </c>
       <c r="BI7" t="inlineStr">
         <is>
-          <t>1;1;0.01;0.2</t>
+          <t>1;1;0.01;0.3</t>
         </is>
       </c>
       <c r="BJ7" t="inlineStr"/>
@@ -1726,14 +1730,18 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>967</v>
+        <v>991</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>992</v>
+      </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>992</v>
+      </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1766,7 +1774,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-1.37</v>
+        <v>-1.18</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1812,10 +1820,10 @@
         </is>
       </c>
       <c r="BC8" t="n">
-        <v>-0.0002</v>
+        <v>-0.003</v>
       </c>
       <c r="BD8" t="n">
-        <v>-0.0002</v>
+        <v>-0.003</v>
       </c>
       <c r="BE8" t="inlineStr">
         <is>
@@ -1828,12 +1836,12 @@
       <c r="BG8" t="inlineStr"/>
       <c r="BH8" t="inlineStr">
         <is>
-          <t>105167;289072.5;86701.25; (10)</t>
+          <t>100321;269897.5;84844.75; (10)</t>
         </is>
       </c>
       <c r="BI8" t="inlineStr">
         <is>
-          <t>1;1;0.01;0.2</t>
+          <t>1;1;0.01;0.3</t>
         </is>
       </c>
       <c r="BJ8" t="inlineStr"/>
@@ -1858,6 +1866,435 @@
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>992</v>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>993</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>993</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>RIZ5</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>MXZ5</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>SiZ5</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>10;60</t>
+        </is>
+      </c>
+      <c r="BC9" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>1;10000</t>
+        </is>
+      </c>
+      <c r="BF9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>100321;269897.5;84844.75; (10)</t>
+        </is>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>1;1;0.01;0.3</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BO9" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>993</v>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>994</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>994</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>RIZ5</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>MXZ5</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>SiZ5</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>10;60</t>
+        </is>
+      </c>
+      <c r="BC10" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>1;10000</t>
+        </is>
+      </c>
+      <c r="BF10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>1;6</t>
+        </is>
+      </c>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>100321;269897.5;84844.75; (10)</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>1;1;0.01;0.3</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BO10" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>994</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>RIZ5</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>MXZ5</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>SiZ5</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>LKZ5</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>10;60</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>1;10000</t>
+        </is>
+      </c>
+      <c r="BF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>100319.5;269891.25;84844.75;60249.95; (10)</t>
+        </is>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>1;1;0.01;0.3</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>2025.04.14 09:00:00</t>
+        </is>
+      </c>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BO11" t="inlineStr">
+        <is>
+          <t>09:00:20-18:50:00 19:05:05-23:50:00</t>
+        </is>
+      </c>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>